<commit_message>
Preserve native wall contacts and align regression fixtures
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -116,8 +116,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E34" totalsRowShown="0">
-  <autoFilter ref="A5:E34"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E35" totalsRowShown="0">
+  <autoFilter ref="A5:E35"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="E10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1967,7 @@
       </c>
       <c r="E11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
@@ -2237,14 +2237,14 @@
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/hive-missions-v131.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2254,24 +2254,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b10e7dfc090367718c6b33263ca08b57bc584531af793cc8f6168966ec788069</t>
+          <t xml:space="preserve">b4538a7e3cd6fa58275a29e8585c52b3788000bbbb61bc39419e5dd6f5756b20</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-story-v160.mjs ; scripts/verify-archive-relay-presentation-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2281,24 +2281,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">b10e7dfc090367718c6b33263ca08b57bc584531af793cc8f6168966ec788069</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-story-v160.mjs ; scripts/verify-archive-relay-presentation-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-v160.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92b77b736978e9bd25a7c01dbf31b44b1c2e8051157357ec72a391a0fa10dc9d</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
@@ -2325,7 +2325,7 @@
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-action-rig-v127.js</t>
+          <t xml:space="preserve">src/motion-tracker-v160.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -2335,24 +2335,24 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f10520f04b4bdf3e84f53e8b61a8bb970e49e3e4a4597b32af3c6a6d40761195</t>
+          <t xml:space="preserve">92b77b736978e9bd25a7c01dbf31b44b1c2e8051157357ec72a391a0fa10dc9d</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
+          <t xml:space="preserve">src/player-action-rig-v127.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -2362,24 +2362,24 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
+          <t xml:space="preserve">f10520f04b4bdf3e84f53e8b61a8bb970e49e3e4a4597b32af3c6a6d40761195</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-body-rig-v125.js</t>
+          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2389,24 +2389,24 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
+          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-body-rig-v125.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2416,24 +2416,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2443,24 +2443,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2470,24 +2470,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2497,24 +2497,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2524,24 +2524,24 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">dc73fb0ad6183e0e4be80e85f525db6b375e3ffe498fec2112a60c491606309d</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Raccorde le bassin, la ceinture, le torse et les jambes dans le même repère de rendu, avec stature et attaches réduites à une enveloppe de conception cohérente et appuis conservés.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2551,42 +2551,69 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">03004ebf7a640eccd537132a5f44d38852f1f3061da5a31dd15754c5abb63e55</t>
+          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V159</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03004ebf7a640eccd537132a5f44d38852f1f3061da5a31dd15754c5abb63e55</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+        </is>
+      </c>
+      <c r="E34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B34" s="0" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V159</t>
         </is>
       </c>
-      <c r="C34" s="0" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">6d9706400fc34044d293a0d54c43396662de77c7e676bc8631df5b4ae287216b</t>
         </is>
       </c>
-      <c r="D34" s="0" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Actualise le shell hors ligne V160 pour charger les modules réellement intégrés et évite de servir un mélange de versions anciennes et nouvelles.</t>
         </is>
       </c>
-      <c r="E34" s="0" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-save-lifecycle-v143.mjs ; scripts/verify-public-release-v86.mjs</t>
         </is>
@@ -20740,17 +20767,17 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres.</t>
+          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre.</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -20765,7 +20792,7 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final.</t>
+          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final. Le contact Jeri adapte le rig existant ; il ne fournit aucun nouvel art synthétique dédié ni animation de franchise certifiée.</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
@@ -20876,7 +20903,7 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
@@ -28150,17 +28177,17 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres.</t>
+          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final.</t>
+          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final. Le contact Jeri adapte le rig existant ; il ne fournit aucun nouvel art synthétique dédié ni animation de franchise certifiée.</t>
         </is>
       </c>
     </row>
@@ -28361,7 +28388,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -28371,7 +28398,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final.</t>
+          <t xml:space="preserve">Correction procédurale de dessins natifs conservés ; enveloppe de conception et mesures de pixels, pas calibration anatomique universelle. Le relevé CMU générique ne retargete aucun personnage de franchise. La collision native reste 42 × 92 unités ; les variantes finales des bras et les comparaisons visuelles avant/après attendent la recette du commit final. Le contact Jeri adapte le rig existant ; il ne fournit aucun nouvel art synthétique dédié ni animation de franchise certifiée.</t>
         </is>
       </c>
     </row>
@@ -28405,7 +28432,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Keep Port Meridien contacts on its painted rung grid
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -116,8 +116,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E35" totalsRowShown="0">
-  <autoFilter ref="A5:E35"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E36" totalsRowShown="0">
+  <autoFilter ref="A5:E36"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -2259,12 +2259,12 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
@@ -2367,19 +2367,19 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2389,24 +2389,24 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-body-rig-v125.js</t>
+          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2416,24 +2416,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
+          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-body-rig-v125.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2443,24 +2443,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2470,24 +2470,24 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2497,24 +2497,24 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2524,24 +2524,24 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2551,24 +2551,24 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses de déplacement et de transit gardent leurs appuis et leur repère commun ; une face physique explicite distingue le contact mural Jeri des barreaux centrés et du plafond, sans modifier les longueurs des membres.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -2578,42 +2578,69 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">03004ebf7a640eccd537132a5f44d38852f1f3061da5a31dd15754c5abb63e55</t>
+          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V159</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03004ebf7a640eccd537132a5f44d38852f1f3061da5a31dd15754c5abb63e55</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+        </is>
+      </c>
+      <c r="E35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B35" s="0" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V159</t>
         </is>
       </c>
-      <c r="C35" s="0" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">6d9706400fc34044d293a0d54c43396662de77c7e676bc8631df5b4ae287216b</t>
         </is>
       </c>
-      <c r="D35" s="0" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Actualise le shell hors ligne V160 pour charger les modules réellement intégrés et évite de servir un mélange de versions anciennes et nouvelles.</t>
         </is>
       </c>
-      <c r="E35" s="0" t="inlineStr">
+      <c r="E36" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-save-lifecycle-v143.mjs ; scripts/verify-public-release-v86.mjs</t>
         </is>
@@ -20767,17 +20794,17 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre.</t>
+          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre. Au Port Méridien, même sous le wrapper spatial de production, le rig conserve les métadonnées du montage natif : pas de 24 pixels et premier barreau à 8 pixels sous le haut de l’échelle, au lieu du montage spatial du vaisseau à 22/11. Les contacts restent à l’intérieur des traverses peintes sans lire les pixels en direct ni déplacer le décor.</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js ; src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
@@ -28177,12 +28204,12 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js ; src/player-body-rig-v125.js ; src/player-locomotion-rig-v129.js ; src/player-modular-rig-v126.js ; src/player-action-rig-v127.js ; src/player-transit-rig-v128.js ; src/player-gait-v133.js ; src/hive-missions-v131.js ; src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre.</t>
+          <t xml:space="preserve">Les pieds, le bassin, la ceinture, le thorax et les épaules de l’arme partagent le même repère de support au lieu de dissocier le haut et le bas du corps. La tête, le casque et le masque utilisent une attache réduite commune ; les hanches projetées sont resserrées. Les longueurs de cuisse/tibia restent rigides, les appuis plantés sont conservés et la cadence suit la distance réelle en marche et jogging. Les raccords de poses, d’échelle, de conduit et de chargement partiel conservent les supports natifs. La poche de recharge suit le tissu de la cuisse éloignée, y compris pendant les poses et le secours de chargement natif, au lieu de rester suspendue à un point vide. Lors d’un chargement incomplet, les sept pièces de jambes disponibles restent procédurales ; si leurs images manquent aussi, les vraies frames natives 4–7 suivent la phase de marche avec leurs propres ancres de semelle. Sur échelle, la posture entière s’écarte du montant pour que la main éloignée reste sur le vrai barreau dans l’enveloppe du coude, sans déplacer les barreaux ni changer les longueurs des membres. Pour le contact mural Jeri, l’identifiant et la face de la surface physique choisissent une posture de prise distincte de l’échelle centrée ; les mains et les pieds plantés visent la vraie face sans projection hors portée, et le plafond garde sa présentation propre. Au Port Méridien, même sous le wrapper spatial de production, le rig conserve les métadonnées du montage natif : pas de 24 pixels et premier barreau à 8 pixels sous le haut de l’échelle, au lieu du montage spatial du vaisseau à 22/11. Les contacts restent à l’intérieur des traverses peintes sans lire les pixels en direct ni déplacer le décor.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
@@ -28388,7 +28415,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Fix campaign persistence and native tracker and weapon inputs
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -116,8 +116,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E36" totalsRowShown="0">
-  <autoFilter ref="A5:E36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AuditV160Table11" displayName="AuditV160Table11" ref="A5:E37" totalsRowShown="0">
+  <autoFilter ref="A5:E37"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="SHA V158"/>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">9f39b1588a8a2316b288481495948586c126494ebecefe779f8e4c90cc7f19f7</t>
+          <t xml:space="preserve">72918e62a99e91e504302834f76e6f9489195299f366f84ee858f850a7272ba1</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Branche les contrôles natifs du détecteur, le mouvement réduit et les retours de la même campagne ; la sauvegarde en mission réutilise le handler réel et le retour après extraction affiche RETOUR À BORD.</t>
+          <t xml:space="preserve">Branche les contrôles natifs, la reprise audio partagée de Q et du bouton sans scan obsolète, et le dernier compte rendu QZ-18 borné au bon plan ; sa préservation et ses lectures utilisent les transactions de sauvegarde natives sans paiement archivé.</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
         </is>
       </c>
       <c r="E10" s="0" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="D11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
         </is>
       </c>
       <c r="E11" s="0" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0fce41555d8a8376d75a0e77f5eddb06bf1ef5548901f3a55ad000f8a3962354</t>
+          <t xml:space="preserve">192432c7cb0aad9d8b3d119cf5f819d031e92f27a8ad0eea8aab02dba2c532a2</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -2082,7 +2082,7 @@
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-consequences.js</t>
+          <t xml:space="preserve">src/archive-relay-state-v122.js</t>
         </is>
       </c>
       <c r="B16" s="0" t="inlineStr">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">359a55917b4cb2cfa2be07485d202cbfc57ca993dbeaaec5097801bda4504f0e</t>
+          <t xml:space="preserve">ccfdc9b9de9bfe30270f12018d450f9cfa69c8e614eb2d4df18d872607abac29</t>
         </is>
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2109,7 +2109,7 @@
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-story-ui-v160.js</t>
+          <t xml:space="preserve">src/campaign-consequences.js</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5872809077adf1f06443997e62834f3b94df62df11b0e4b9a717e4ba07c68946</t>
+          <t xml:space="preserve">359a55917b4cb2cfa2be07485d202cbfc57ca993dbeaaec5097801bda4504f0e</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -2136,7 +2136,7 @@
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-story-v160.js</t>
+          <t xml:space="preserve">src/campaign-story-ui-v160.js</t>
         </is>
       </c>
       <c r="B18" s="0" t="inlineStr">
@@ -2146,12 +2146,12 @@
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">12bad86f8d591efe2e8aaa898bb7f26ceff38528687ad174731f1840cd11d37c</t>
+          <t xml:space="preserve">94c8dea45e869e308f72e9905530bf0c2a1ab584d7951f906a3747c73a8a96e4</t>
         </is>
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -2163,7 +2163,7 @@
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/game-production-base.js</t>
+          <t xml:space="preserve">src/campaign-story-v160.js</t>
         </is>
       </c>
       <c r="B19" s="0" t="inlineStr">
@@ -2173,24 +2173,24 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">95b136fcc0caade82a784522dcedc635d6acb2ad91ba6517c6d07fb36ca89793</t>
+          <t xml:space="preserve">aa458b8917aa1454e7c8e9c3a035428e6b3704f564b44e1aa0e7dc6d89d73d4c</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-story-v160.mjs ; scripts/verify-archive-relay-presentation-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/game-v52-level-runtime.js</t>
+          <t xml:space="preserve">src/game-production-base.js</t>
         </is>
       </c>
       <c r="B20" s="0" t="inlineStr">
@@ -2200,12 +2200,12 @@
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f394cdc77d4684846cbfb5552ec950f4ba9948d75a09091177627ae7763112c4</t>
+          <t xml:space="preserve">95b136fcc0caade82a784522dcedc635d6acb2ad91ba6517c6d07fb36ca89793</t>
         </is>
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -2217,7 +2217,7 @@
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
+          <t xml:space="preserve">src/game-v52-level-runtime.js</t>
         </is>
       </c>
       <c r="B21" s="0" t="inlineStr">
@@ -2227,24 +2227,24 @@
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
+          <t xml:space="preserve">f394cdc77d4684846cbfb5552ec950f4ba9948d75a09091177627ae7763112c4</t>
         </is>
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/hive-missions-v131.js</t>
+          <t xml:space="preserve">src/held-weapon-renderer-v125.js</t>
         </is>
       </c>
       <c r="B22" s="0" t="inlineStr">
@@ -2254,24 +2254,24 @@
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b4538a7e3cd6fa58275a29e8585c52b3788000bbbb61bc39419e5dd6f5756b20</t>
+          <t xml:space="preserve">bf20b93457fbd7d6296acf66aacf1175698d4d68092c1297465df6a64dcaba5f</t>
         </is>
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
         </is>
       </c>
       <c r="E22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
+          <t xml:space="preserve">src/hive-missions-v131.js</t>
         </is>
       </c>
       <c r="B23" s="0" t="inlineStr">
@@ -2281,24 +2281,24 @@
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">b10e7dfc090367718c6b33263ca08b57bc584531af793cc8f6168966ec788069</t>
+          <t xml:space="preserve">b4538a7e3cd6fa58275a29e8585c52b3788000bbbb61bc39419e5dd6f5756b20</t>
         </is>
       </c>
       <c r="D23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dossier QZ18 relie préparation, mission réelle, pièces persistantes et débrief de la même opération, sans récompenser la lecture ni remplacer les conséquences natives.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-campaign-story-v160.mjs ; scripts/verify-archive-relay-presentation-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
+          <t xml:space="preserve">src/mission-insertion-ui-v62.js</t>
         </is>
       </c>
       <c r="B24" s="0" t="inlineStr">
@@ -2308,24 +2308,24 @@
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
+          <t xml:space="preserve">70fcb59b28ba6f48a974fca4195cd685a9fc2e178efead7e56a64e180b3b6ab2</t>
         </is>
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
+          <t xml:space="preserve">scripts/verify-campaign-story-v160.mjs ; scripts/verify-archive-relay-presentation-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/motion-tracker-v160.js</t>
+          <t xml:space="preserve">src/motion-tracker-display-v160.js</t>
         </is>
       </c>
       <c r="B25" s="0" t="inlineStr">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92b77b736978e9bd25a7c01dbf31b44b1c2e8051157357ec72a391a0fa10dc9d</t>
+          <t xml:space="preserve">0b82e164c2ffd3439317e5ccef3c5892f1f920932072111cc5d1b7958682ad4d</t>
         </is>
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les observations, le balayage et le HUD du détecteur emploient des échos mobiles bornés au repère actif plutôt qu’un relevé omniscient des ennemis vivants.</t>
+          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -2352,7 +2352,7 @@
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-action-rig-v127.js</t>
+          <t xml:space="preserve">src/motion-tracker-v160.js</t>
         </is>
       </c>
       <c r="B26" s="0" t="inlineStr">
@@ -2362,24 +2362,24 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">f10520f04b4bdf3e84f53e8b61a8bb970e49e3e4a4597b32af3c6a6d40761195</t>
+          <t xml:space="preserve">92b77b736978e9bd25a7c01dbf31b44b1c2e8051157357ec72a391a0fa10dc9d</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
+          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-motion-tracker-v160.mjs</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
+          <t xml:space="preserve">src/player-action-rig-v127.js</t>
         </is>
       </c>
       <c r="B27" s="0" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
+          <t xml:space="preserve">f10520f04b4bdf3e84f53e8b61a8bb970e49e3e4a4597b32af3c6a6d40761195</t>
         </is>
       </c>
       <c r="D27" s="0" t="inlineStr">
@@ -2406,7 +2406,7 @@
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
+          <t xml:space="preserve">src/player-appearance-hub-v126.js</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -2416,24 +2416,24 @@
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
+          <t xml:space="preserve">584adbd984e3f4f07846043ead8bf0c5f87c2f568e508c38318996e47a046cc8</t>
         </is>
       </c>
       <c r="D28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-body-rig-v125.js</t>
+          <t xml:space="preserve">src/player-arm-constraints-v160.js</t>
         </is>
       </c>
       <c r="B29" s="0" t="inlineStr">
@@ -2443,24 +2443,24 @@
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
+          <t xml:space="preserve">1c502fb559aabc20a603cb7fe220640986409a22c7d00831ff96d4277291922c</t>
         </is>
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
         </is>
       </c>
       <c r="E29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
         </is>
       </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-gait-v133.js</t>
+          <t xml:space="preserve">src/player-body-rig-v125.js</t>
         </is>
       </c>
       <c r="B30" s="0" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
+          <t xml:space="preserve">401f81aaf0b2f1ab3b90353486782aa755fb54fd16084a5beda964c5d6c8a1df</t>
         </is>
       </c>
       <c r="D30" s="0" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
+          <t xml:space="preserve">src/player-gait-v133.js</t>
         </is>
       </c>
       <c r="B31" s="0" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
+          <t xml:space="preserve">8210c7f89a0db7d9e3a0f2fb0138d9819bead4ed1df83d8aa8eb97d1bb32c310</t>
         </is>
       </c>
       <c r="D31" s="0" t="inlineStr">
@@ -2514,7 +2514,7 @@
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
+          <t xml:space="preserve">src/player-human-proportions-v160.js</t>
         </is>
       </c>
       <c r="B32" s="0" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
+          <t xml:space="preserve">e9dda6a8c2a79947eb6ba87461078bcc6be0b907bd7e04492f24927a842341e1</t>
         </is>
       </c>
       <c r="D32" s="0" t="inlineStr">
@@ -2541,7 +2541,7 @@
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
+          <t xml:space="preserve">src/player-locomotion-rig-v129.js</t>
         </is>
       </c>
       <c r="B33" s="0" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
+          <t xml:space="preserve">a7401d90b4dd0a6ef9c7da2322bab03f6fb175618428b66357e6fbf1ac3ac957</t>
         </is>
       </c>
       <c r="D33" s="0" t="inlineStr">
@@ -2568,7 +2568,7 @@
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
+          <t xml:space="preserve">src/player-modular-rig-v126.js</t>
         </is>
       </c>
       <c r="B34" s="0" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
+          <t xml:space="preserve">cbf671c6d508e40dbc38d84f0a871cb840b94aa773a5bcd81eb43109b51f7e2f</t>
         </is>
       </c>
       <c r="D34" s="0" t="inlineStr">
@@ -2595,7 +2595,7 @@
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+          <t xml:space="preserve">src/player-transit-rig-v128.js</t>
         </is>
       </c>
       <c r="B35" s="0" t="inlineStr">
@@ -2605,42 +2605,69 @@
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">03004ebf7a640eccd537132a5f44d38852f1f3061da5a31dd15754c5abb63e55</t>
+          <t xml:space="preserve">872cb530d903bab7cb0b9cb26da9652926f9e588c98c8a88ad9c034b45814613</t>
         </is>
       </c>
       <c r="D35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">La prévision pure du corps après déclenchement, le raccord mains/arme et les gardes natives de tir/cycles évitent une pose impossible ou un prélèvement de ressource avant un tir refusé.</t>
+          <t xml:space="preserve">Les poses gardent leur repère et leurs vrais supports : face physique du mur Jeri, grille centrée des échelles et origine/pas réellement peints par le montage spécifique du Port Méridien, sans changer les os.</t>
         </is>
       </c>
       <c r="E35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+          <t xml:space="preserve">scripts/verify-player-human-coherence-v160.mjs ; scripts/verify-player-body-alignment-v142.mjs ; scripts/verify-jeri-surface-motion-v135.mjs ; scripts/verify-player-climb-contacts-v139.mjs ; scripts/verify-human-gait-v133.mjs ; scripts/verify-human-motion-v136.mjs ; scripts/verify-player-appearance-runtime-v126.mjs</t>
         </is>
       </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">src/player-weapon-runtime-v125.js</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non épinglé en V159</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8f18c50f16c5f00f9dae9c3210ef51bbe4671efce1512d5f0f86ae95b9ab6342</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">La prévision pure et les gardes natives refusent les tirs obstrués avant ressources ; les charges et rafales conservent le côté de leur visée différée au lieu de simuler un corps tourné à l’opposé.</t>
+        </is>
+      </c>
+      <c r="E36" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/verify-held-weapon-v125.mjs ; scripts/verify-player-weapon-rig-v125.mjs ; scripts/verify-weapon-actions-v131.mjs ; scripts/verify-player-runtime-v124.mjs ; scripts/verify-audit-v143.mjs ; scripts/verify-destructible-scenery-v130.mjs ; scripts/verify-forge-mission-v141.mjs ; scripts/verify-placeables-extension-v132.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">sw.js</t>
         </is>
       </c>
-      <c r="B36" s="0" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Non épinglé en V159</t>
         </is>
       </c>
-      <c r="C36" s="0" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">6d9706400fc34044d293a0d54c43396662de77c7e676bc8631df5b4ae287216b</t>
         </is>
       </c>
-      <c r="D36" s="0" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Actualise le shell hors ligne V160 pour charger les modules réellement intégrés et évite de servir un mélange de versions anciennes et nouvelles.</t>
         </is>
       </c>
-      <c r="E36" s="0" t="inlineStr">
+      <c r="E37" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">scripts/verify-save-lifecycle-v143.mjs ; scripts/verify-public-release-v86.mjs</t>
         </is>
@@ -20857,7 +20884,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu.</t>
+          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -20920,7 +20947,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le solveur maintient les mains dans une enveloppe de conception réalisable, avec des zones de poignée, avant-main et port de service qui évitent la singularité près de l’épaule, et une portée d’épaule mesurée depuis le vrai torse. Le corps final V129 est résolu avant le canon et l’origine du tir. Lors d’un obstacle réel, la rétraction recalcule l’arme rigide et les mains sans déplacer la poche du corps pendant la recharge. Un aperçu pur de la pose après déclenchement, blessure et recul prévoit le vrai cadrage avant de dépenser une ressource ou de lancer un cycle. La projection du curseur peut être consultée sans mutation ; les gardes de tir et de commit refusent les cycles obstrués avant leur consommation. Le guide d’obstruction suit la garde physique courante : un ancien flag de pose ne bloque plus un canon réellement dégagé après un peek, et un vrai contact au mur conserve le refus avant ressources.</t>
+          <t xml:space="preserve">Le solveur maintient les mains dans une enveloppe de conception réalisable, avec des zones de poignée, avant-main et port de service qui évitent la singularité près de l’épaule, et une portée d’épaule mesurée depuis le vrai torse. Le corps final V129 est résolu avant le canon et l’origine du tir. Lors d’un obstacle réel, la rétraction recalcule l’arme rigide et les mains sans déplacer la poche du corps pendant la recharge. Un aperçu pur de la pose après déclenchement, blessure et recul prévoit le vrai cadrage avant de dépenser une ressource ou de lancer un cycle. La projection du curseur peut être consultée sans mutation ; les gardes de tir et de commit refusent les cycles obstrués avant leur consommation. Le guide d’obstruction suit la garde physique courante : un ancien flag de pose ne bloque plus un canon réellement dégagé après un peek, et un vrai contact au mur conserve le refus avant ressources. Pour les tirs différés de charge ou de rafale, l’aperçu conserve l’orientation explicitement fournie ; si la visée stockée ne contient que x/y, son sens horizontal détermine le côté du corps, avec repli sur l’orientation de l’acteur pour une visée verticale. L’aperçu ne modifie pas cette visée.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -20983,12 +21010,12 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ».</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-story-v160.js ; src/campaign-story-ui-v160.js ; src/mission-insertion-ui-v62.js ; src/campaign-consequences.js ; src/archive-relay-presentation-v160.js ; src/archive-relay-runtime-v122.js ; mission-insertion-v62.css</t>
+          <t xml:space="preserve">src/campaign-story-v160.js ; src/campaign-story-ui-v160.js ; src/mission-insertion-ui-v62.js ; src/campaign-consequences.js ; src/archive-relay-presentation-v160.js ; src/archive-relay-runtime-v122.js ; mission-insertion-v62.css ; src/archive-relay-state-v122.js</t>
         </is>
       </c>
       <c r="F9" s="0" t="inlineStr">
@@ -22845,7 +22872,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Green display with forward fan sector, arc markings and a luminous unclassified point. ; A lower-left distance number is visible; the screenshot reads0.59 without establishing a world-unit conversion. ; Side indicators and a left edge rectangular marker are visible.</t>
+          <t xml:space="preserve">Green display with forward fan sector, arc markings and a luminous unclassified point. ; A lower-left distance number is visible; the screenshot reads 0.59 without establishing a world-unit conversion. ; Side indicators and a left edge rectangular marker are visible.</t>
         </is>
       </c>
       <c r="I7" s="0" t="inlineStr">
@@ -23029,12 +23056,12 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extracted text line23 synopsis; no film frames recovered</t>
+          <t xml:space="preserve">Extracted text line 23 synopsis; no film frames recovered</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ripley returns from hypersleep after57years; lost contact with colonists leads to a military expedition.</t>
+          <t xml:space="preserve">Ripley returns from hypersleep after 57 years; lost contact with colonists leads to a military expedition.</t>
         </is>
       </c>
       <c r="I10" s="0" t="inlineStr">
@@ -23097,7 +23124,7 @@
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">The official montage advertises Pathogen; one environment establishing shot is identified at1.001s.</t>
+          <t xml:space="preserve">The official montage advertises Pathogen; one environment establishing shot is identified at 1.001 s.</t>
         </is>
       </c>
       <c r="I11" s="0" t="inlineStr">
@@ -23155,7 +23182,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Project baseline4fc9da8, generated adapted sprite parts</t>
+          <t xml:space="preserve">Project baseline 4fc9da8, generated adapted sprite parts</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -23266,7 +23293,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminator2D: NO FATE</t>
+          <t xml:space="preserve">Terminator 2D: NO FATE</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -23329,7 +23356,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">CMU Graphics Lab Motion Capture Database — subject02,trial01,walk</t>
+          <t xml:space="preserve">CMU Graphics Lab Motion Capture Database — subject 02, trial 01, walk</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -23344,7 +23371,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bruce Hahne MotionBuilder-friendly BVH2010 release; T-pose estimated and prepended</t>
+          <t xml:space="preserve">Bruce Hahne MotionBuilder-friendly BVH 2010 release; T-pose estimated and prepended</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -23354,7 +23381,7 @@
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">One walk capture by one performer, not universal joint limits or a canonical franchise animation. ; READMEFIRST explicitly warns CMU joint calibration/T-pose are guessed and source motion may contain impossible head angles/noise. ; Frame0 is synthetic added T-pose; excluded from motion extrema. ; Knee flexion measured from 3D segment geometry; hip-like value uses world vertical/travel plane, not calibrated anatomical pelvis joint angle. ; Source game speed, phase, mappingnear/far vsleft/right differ; no1:1 certification or direct targetdegreeconstraint. ; Sourceunits, subject anthropometry and marker calibration not established. ; This source does not certify an Aliens,Terminator or other franchise animation. ; Finger/thumb motion is not captured according to the README; cannot validate weapon grip animation. ; No BVH,raw capture,PNG or private trace is proposed for the public repository.</t>
+          <t xml:space="preserve">One walk capture by one performer, not universal joint limits or a canonical franchise animation. ; READMEFIRST explicitly warns CMU joint calibration/T-pose are guessed and source motion may contain impossible head angles/noise. ; Frame 0 is synthetic added T-pose; excluded from motion extrema. ; Knee flexion measured from 3D segment geometry; hip-like value uses world vertical/travel plane, not calibrated anatomical pelvis joint angle. ; Source game speed, phase, mapping near/far vs left/right differ; no 1:1 certification or direct target degree constraint. ; Source units, subject anthropometry and marker calibration not established. ; This source does not certify an Aliens, Terminator or other franchise animation. ; Finger/thumb motion is not captured according to the README; cannot validate weapon grip animation. ; No BVH, raw capture, PNG or private trace is proposed for the public repository.</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
@@ -23464,7 +23491,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Neutral left/right next to the same human NPC and floor. ; At leastone full slow walking cycle left/right, running cycle, brake and restart. ; Crouch idle/move, jump ascent/apex/landing, ladder step and vent entry/exit. ; Same camera zoom, viewport, outfit, neutral pose and known Save-picker fixture before/after.</t>
+          <t xml:space="preserve">Neutral left/right next to the same human NPC and floor. ; At least one full slow walking cycle left/right, running cycle, brake and restart. ; Crouch idle/move, jump ascent/apex/landing, ladder step and vent entry/exit. ; Same camera zoom, viewport, outfit, neutral pose and known Save-picker fixture before/after.</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -23474,7 +23501,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">No detached waist, reversed knee, below-floor sole or visibly rescaled leg across postures. ; Numeric constraints are engineering plausibility checks; external anatomical1:1 remains unapproved.</t>
+          <t xml:space="preserve">No detached waist, reversed knee, below-floor sole or visibly rescaled leg across postures. ; Numeric constraints are engineering plausibility checks; external anatomical 1:1 remains unapproved.</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">
@@ -28236,7 +28263,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu.</t>
+          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -28263,7 +28290,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le solveur maintient les mains dans une enveloppe de conception réalisable, avec des zones de poignée, avant-main et port de service qui évitent la singularité près de l’épaule, et une portée d’épaule mesurée depuis le vrai torse. Le corps final V129 est résolu avant le canon et l’origine du tir. Lors d’un obstacle réel, la rétraction recalcule l’arme rigide et les mains sans déplacer la poche du corps pendant la recharge. Un aperçu pur de la pose après déclenchement, blessure et recul prévoit le vrai cadrage avant de dépenser une ressource ou de lancer un cycle. La projection du curseur peut être consultée sans mutation ; les gardes de tir et de commit refusent les cycles obstrués avant leur consommation. Le guide d’obstruction suit la garde physique courante : un ancien flag de pose ne bloque plus un canon réellement dégagé après un peek, et un vrai contact au mur conserve le refus avant ressources.</t>
+          <t xml:space="preserve">Le solveur maintient les mains dans une enveloppe de conception réalisable, avec des zones de poignée, avant-main et port de service qui évitent la singularité près de l’épaule, et une portée d’épaule mesurée depuis le vrai torse. Le corps final V129 est résolu avant le canon et l’origine du tir. Lors d’un obstacle réel, la rétraction recalcule l’arme rigide et les mains sans déplacer la poche du corps pendant la recharge. Un aperçu pur de la pose après déclenchement, blessure et recul prévoit le vrai cadrage avant de dépenser une ressource ou de lancer un cycle. La projection du curseur peut être consultée sans mutation ; les gardes de tir et de commit refusent les cycles obstrués avant leur consommation. Le guide d’obstruction suit la garde physique courante : un ancien flag de pose ne bloque plus un canon réellement dégagé après un peek, et un vrai contact au mur conserve le refus avant ressources. Pour les tirs différés de charge ou de rafale, l’aperçu conserve l’orientation explicitement fournie ; si la visée stockée ne contient que x/y, son sens horizontal détermine le côté du corps, avec repli sur l’orientation de l’acteur pour une visée verticale. L’aperçu ne modifie pas cette visée.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -28285,12 +28312,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">src/campaign-story-v160.js ; src/campaign-story-ui-v160.js ; src/mission-insertion-ui-v62.js ; src/campaign-consequences.js ; src/archive-relay-presentation-v160.js ; src/archive-relay-runtime-v122.js ; mission-insertion-v62.css</t>
+          <t xml:space="preserve">src/campaign-story-v160.js ; src/campaign-story-ui-v160.js ; src/mission-insertion-ui-v62.js ; src/campaign-consequences.js ; src/archive-relay-presentation-v160.js ; src/archive-relay-runtime-v122.js ; mission-insertion-v62.css ; src/archive-relay-state-v122.js</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ».</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Preserve QZ-18 reading archive after normalized saves
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -2016,7 +2016,7 @@
       </c>
       <c r="D13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E13" s="0" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="D14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E14" s="0" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E16" s="0" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="D18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E18" s="0" t="inlineStr">
@@ -2173,12 +2173,12 @@
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">aa458b8917aa1454e7c8e9c3a035428e6b3704f564b44e1aa0e7dc6d89d73d4c</t>
+          <t xml:space="preserve">649bb76d681b3d162d9966163becf1e65e9b40f3b3e5c6216dd6cc17acb8cd4c</t>
         </is>
       </c>
       <c r="D19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E19" s="0" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le dernier compte rendu QZ-18 reste borné et lié au dossier de la même opération après une autre sortie ; son affichage suit le plan choisi, ses lectures ne paient jamais et les insertions ordinaires conservent leurs interactions.</t>
+          <t xml:space="preserve">Le compte rendu QZ-18 reste lié au dossier de la même opération ; ses lectures après normalisation actualisent ensemble les deux registres en conservant les seules dates attestées, sans paiement.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">
@@ -21010,7 +21010,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu.</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu.</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Keep keyboard focus when reading the QZ-18 debrief
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -1822,7 +1822,7 @@
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">72918e62a99e91e504302834f76e6f9489195299f366f84ee858f850a7272ba1</t>
+          <t xml:space="preserve">6b24708217b760d34181adb36525f62348ca5b9522368044c839cfa31be0c0d6</t>
         </is>
       </c>
       <c r="D6" s="0" t="inlineStr">
@@ -21010,7 +21010,7 @@
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée.</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée. Après reconstruction du plan, la question activée retrouve le focus clavier sans déplacement de page, y compris en relecture.</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée.</t>
+          <t xml:space="preserve">« Le dernier relais » approfondit QZ-18/Lethe dans l’opération special-archive-relay : cinq phases dialoguées avec portraits natifs, avec l’incident natif lorsqu’il est présent, choix de préparation technique ou de prévention à bord, six pièces persistantes et retour rattaché au même identifiant d’opération. Les retombées de recherche ou de moral exigent extraction native et dossier complet ; lecture/relecture ne récompensent jamais, et les blessures/échecs restent réels. Le déploiement emploie le même renderer QZ-18 que la mission ; les props réutilisent cinq atlas admis, au contact des vraies ancres, en 2D intégrale sans ajouter de collision. Les contrôles de sauvegarde en mission et de retour après extraction utilisent les handlers natifs ; le retour est libellé « RETOUR À BORD ». Le dernier compte rendu QZ-18 est conservé avec son dossier, accessible après une autre opération ; ce retour compact et borné garde son identifiant, son résultat, son protocole et son reçu de lecture/paiement. Il est affiché uniquement dans le plan QZ-18 ; le paiement lit seulement le résultat natif courant, jamais le retour archivé. Les insertions ordinaires retrouvent leurs interactions contextuelles et le cadrage des illustrations suit la progression persistée de la phase, sans redémarrer une animation à chaque rendu. Après normalisation native de la sauvegarde, les six lectures mettent à jour le bilan courant et son archive durable ensemble. Les dates proviennent seulement du retour validé de cette même opération, ou du dossier natif correspondant pour une ancienne victoire ; aucune date courante ni récompense supplémentaire n’est créée. Après reconstruction du plan, la question activée retrouve le focus clavier sans déplacement de page, y compris en relecture.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Track native hive bodies and supply anatomy QA defaults
</commit_message>
<xml_diff>
--- a/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
+++ b/docs/forge/xeno-trials/XENO_TRIALS_SUIVI_V160.xlsx
@@ -1881,7 +1881,7 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
+          <t xml:space="preserve">Les castes physiques du registre natif des missions de ruche actives utilisent les mêmes mesures de mouvement et les mêmes gardes que les autres corps ; ni leur loyauté ni leur recrutement ne sont révélés.</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="D20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
+          <t xml:space="preserve">Les castes physiques du registre natif des missions de ruche actives utilisent les mêmes mesures de mouvement et les mêmes gardes que les autres corps ; ni leur loyauté ni leur recrutement ne sont révélés.</t>
         </is>
       </c>
       <c r="E20" s="0" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
+          <t xml:space="preserve">Les castes physiques du registre natif des missions de ruche actives utilisent les mêmes mesures de mouvement et les mêmes gardes que les autres corps ; ni leur loyauté ni leur recrutement ne sont révélés.</t>
         </is>
       </c>
       <c r="E21" s="0" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
+          <t xml:space="preserve">Les castes physiques du registre natif des missions de ruche actives utilisent les mêmes mesures de mouvement et les mêmes gardes que les autres corps ; ni leur loyauté ni leur recrutement ne sont révélés.</t>
         </is>
       </c>
       <c r="E25" s="0" t="inlineStr">
@@ -2362,12 +2362,12 @@
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">92b77b736978e9bd25a7c01dbf31b44b1c2e8051157357ec72a391a0fa10dc9d</t>
+          <t xml:space="preserve">cbe9be7d43640a9a4f52b8ad34a8cedce7a8cf90f5ff7eda3a477c2cb038216f</t>
         </is>
       </c>
       <c r="D26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les échos mobiles restent bornés au repère actif ; Q et le bouton natif partagent une reprise audio admise dans le geste, avec rejet des demandes devenues obsolètes avant consultation.</t>
+          <t xml:space="preserve">Les castes physiques du registre natif des missions de ruche actives utilisent les mêmes mesures de mouvement et les mêmes gardes que les autres corps ; ni leur loyauté ni leur recrutement ne sont révélés.</t>
         </is>
       </c>
       <c r="E26" s="0" t="inlineStr">
@@ -20884,7 +20884,7 @@
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif.</t>
+          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif. Dans une mission de ruche active, les castes physiques du registre natif hiveActorsV131 participent au même échantillonnage de déplacement, sans distinction de loyauté ou de recrutement. Leurs échos restent anonymes et suivent les mêmes règles de vie, de scène et de disparition.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -28263,7 +28263,7 @@
       </c>
       <c r="D24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif.</t>
+          <t xml:space="preserve">Q active la capacité native de détection à 900 unités du jeu : contacts de positions réellement mobiles dans le même repère/pont, balayage, échos datés et expiration. L’écran en coupe 2D ne révèle ni camp, espèce ou boss ; alliés, ennemis et conduits projetés ne sont suivis que sur mouvement mesuré. Bip et bruit tactique local suivent le temps actif après activation ; pauses, générations et changements de repère ne créent pas de dette de mouvement. Sur écran étroit, le boîtier compact se place d’après le corps et la caméra et affiche une portée relative sans attribuer des mètres aux unités du jeu. À bord, Q et le bouton natif du détecteur partagent la même activation, y compris au clavier focalisé et au clic assistif. Le déverrouillage audio commence dans le geste ; seule une reprise audio audible et suspendue retarde la consultation, puis l’identité du joueur, du propriétaire, de la génération, du repère et de l’impulsion est revérifiée. Un son muet, absent ou refusé laisse le gameplay disponible ; une demande devenue obsolète ne déclenche aucun scan tardif. Dans une mission de ruche active, les castes physiques du registre natif hiveActorsV131 participent au même échantillonnage de déplacement, sans distinction de loyauté ou de recrutement. Leurs échos restent anonymes et suivent les mêmes règles de vie, de scène et de disparition.</t>
         </is>
       </c>
       <c r="E24" s="0" t="inlineStr">

</xml_diff>